<commit_message>
Modelo financiero: separar coste fijo (alquiler+suministros) de personal; nombres reales en CapTable
</commit_message>
<xml_diff>
--- a/entregables/LEGION_modelo_financiero_valoracion_v1.xlsx
+++ b/entregables/LEGION_modelo_financiero_valoracion_v1.xlsx
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="G6" s="97">
-        <f>(Inputs!$B$16+Inputs!$B$17+Inputs!$C$30)/(Inputs!$C$27/(1+Inputs!$B$12)-Inputs!$C$29)</f>
+        <f>(Inputs!$B$16+Inputs!$B$17+Inputs!$B$36+Inputs!$C$30)/(Inputs!$C$27/(1+Inputs!$B$12)-Inputs!$C$29)</f>
         <v/>
       </c>
       <c r="H6" t="inlineStr">
@@ -3183,11 +3183,11 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Coste fijo operativo mensual objetivo</t>
+          <t>Alquiler + IVA + suministros (sin personal)</t>
         </is>
       </c>
       <c r="B16" s="104" t="n">
-        <v>9000</v>
+        <v>4650</v>
       </c>
       <c r="C16" s="15" t="str"/>
       <c r="D16" s="15" t="str"/>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="F16" s="37" t="inlineStr">
         <is>
-          <t>Real estimado: alquiler (2.600) + personal minimo (Sergi+2) + servicios/seguros/gestoria.</t>
+          <t>Real: 2.600 alquiler + 21% IVA (3.146) + suministros luz/agua/seguros estimados (~1.500). El personal va aparte (filas 36-38).</t>
         </is>
       </c>
     </row>
@@ -3628,13 +3628,64 @@
       <c r="F35" s="38" t="n"/>
     </row>
     <row r="36">
-      <c r="F36" s="38" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Personal mensual - meses 1 a 12 (equipo mínimo)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>€/mes</t>
+        </is>
+      </c>
+      <c r="F36" s="38" t="inlineStr">
+        <is>
+          <t>Real: administrador+trabajador (Sergi) + 2 empleados. ~60.000 €/año. Limpieza externalizada, no incluida.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="F37" s="38" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Personal mensual - meses 13 a 24</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>€/mes</t>
+        </is>
+      </c>
+      <c r="F37" s="38" t="inlineStr">
+        <is>
+          <t>Crecimiento de equipo con el volumen de socios. ~78.000 €/año.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="F38" s="38" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Personal mensual - meses 25 a 36</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>7900</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>€/mes</t>
+        </is>
+      </c>
+      <c r="F38" s="38" t="inlineStr">
+        <is>
+          <t>Equipo estabilizado. ~95.000 €/año.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="F39" s="38" t="n"/>
@@ -4325,7 +4376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4428,6 +4479,11 @@
           <t>Nota</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="97" t="n">
@@ -4466,7 +4522,7 @@
         <v/>
       </c>
       <c r="J4" s="98">
-        <f>E4-F4-G4-H4-I4</f>
+        <f>E4-F4-G4-H4-I4-N4</f>
         <v/>
       </c>
       <c r="K4" s="109">
@@ -4475,6 +4531,10 @@
       </c>
       <c r="L4" s="98">
         <f>SUM($J$4:J4)</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>IF(A4&lt;=12,Inputs!$B$36,IF(A4&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4515,7 +4575,7 @@
         <v/>
       </c>
       <c r="J5" s="98">
-        <f>E5-F5-G5-H5-I5</f>
+        <f>E5-F5-G5-H5-I5-N5</f>
         <v/>
       </c>
       <c r="K5" s="109">
@@ -4524,6 +4584,10 @@
       </c>
       <c r="L5" s="98">
         <f>SUM($J$4:J5)</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>IF(A5&lt;=12,Inputs!$B$36,IF(A5&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4564,7 +4628,7 @@
         <v/>
       </c>
       <c r="J6" s="98">
-        <f>E6-F6-G6-H6-I6</f>
+        <f>E6-F6-G6-H6-I6-N6</f>
         <v/>
       </c>
       <c r="K6" s="109">
@@ -4573,6 +4637,10 @@
       </c>
       <c r="L6" s="98">
         <f>SUM($J$4:J6)</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f>IF(A6&lt;=12,Inputs!$B$36,IF(A6&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4613,7 +4681,7 @@
         <v/>
       </c>
       <c r="J7" s="98">
-        <f>E7-F7-G7-H7-I7</f>
+        <f>E7-F7-G7-H7-I7-N7</f>
         <v/>
       </c>
       <c r="K7" s="109">
@@ -4622,6 +4690,10 @@
       </c>
       <c r="L7" s="98">
         <f>SUM($J$4:J7)</f>
+        <v/>
+      </c>
+      <c r="N7">
+        <f>IF(A7&lt;=12,Inputs!$B$36,IF(A7&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4662,7 +4734,7 @@
         <v/>
       </c>
       <c r="J8" s="98">
-        <f>E8-F8-G8-H8-I8</f>
+        <f>E8-F8-G8-H8-I8-N8</f>
         <v/>
       </c>
       <c r="K8" s="109">
@@ -4671,6 +4743,10 @@
       </c>
       <c r="L8" s="98">
         <f>SUM($J$4:J8)</f>
+        <v/>
+      </c>
+      <c r="N8">
+        <f>IF(A8&lt;=12,Inputs!$B$36,IF(A8&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4711,7 +4787,7 @@
         <v/>
       </c>
       <c r="J9" s="98">
-        <f>E9-F9-G9-H9-I9</f>
+        <f>E9-F9-G9-H9-I9-N9</f>
         <v/>
       </c>
       <c r="K9" s="109">
@@ -4720,6 +4796,10 @@
       </c>
       <c r="L9" s="98">
         <f>SUM($J$4:J9)</f>
+        <v/>
+      </c>
+      <c r="N9">
+        <f>IF(A9&lt;=12,Inputs!$B$36,IF(A9&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4760,7 +4840,7 @@
         <v/>
       </c>
       <c r="J10" s="98">
-        <f>E10-F10-G10-H10-I10</f>
+        <f>E10-F10-G10-H10-I10-N10</f>
         <v/>
       </c>
       <c r="K10" s="109">
@@ -4769,6 +4849,10 @@
       </c>
       <c r="L10" s="98">
         <f>SUM($J$4:J10)</f>
+        <v/>
+      </c>
+      <c r="N10">
+        <f>IF(A10&lt;=12,Inputs!$B$36,IF(A10&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4809,7 +4893,7 @@
         <v/>
       </c>
       <c r="J11" s="98">
-        <f>E11-F11-G11-H11-I11</f>
+        <f>E11-F11-G11-H11-I11-N11</f>
         <v/>
       </c>
       <c r="K11" s="109">
@@ -4818,6 +4902,10 @@
       </c>
       <c r="L11" s="98">
         <f>SUM($J$4:J11)</f>
+        <v/>
+      </c>
+      <c r="N11">
+        <f>IF(A11&lt;=12,Inputs!$B$36,IF(A11&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4858,7 +4946,7 @@
         <v/>
       </c>
       <c r="J12" s="98">
-        <f>E12-F12-G12-H12-I12</f>
+        <f>E12-F12-G12-H12-I12-N12</f>
         <v/>
       </c>
       <c r="K12" s="109">
@@ -4867,6 +4955,10 @@
       </c>
       <c r="L12" s="98">
         <f>SUM($J$4:J12)</f>
+        <v/>
+      </c>
+      <c r="N12">
+        <f>IF(A12&lt;=12,Inputs!$B$36,IF(A12&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4907,7 +4999,7 @@
         <v/>
       </c>
       <c r="J13" s="98">
-        <f>E13-F13-G13-H13-I13</f>
+        <f>E13-F13-G13-H13-I13-N13</f>
         <v/>
       </c>
       <c r="K13" s="109">
@@ -4916,6 +5008,10 @@
       </c>
       <c r="L13" s="98">
         <f>SUM($J$4:J13)</f>
+        <v/>
+      </c>
+      <c r="N13">
+        <f>IF(A13&lt;=12,Inputs!$B$36,IF(A13&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -4956,7 +5052,7 @@
         <v/>
       </c>
       <c r="J14" s="98">
-        <f>E14-F14-G14-H14-I14</f>
+        <f>E14-F14-G14-H14-I14-N14</f>
         <v/>
       </c>
       <c r="K14" s="109">
@@ -4965,6 +5061,10 @@
       </c>
       <c r="L14" s="98">
         <f>SUM($J$4:J14)</f>
+        <v/>
+      </c>
+      <c r="N14">
+        <f>IF(A14&lt;=12,Inputs!$B$36,IF(A14&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5005,7 +5105,7 @@
         <v/>
       </c>
       <c r="J15" s="98">
-        <f>E15-F15-G15-H15-I15</f>
+        <f>E15-F15-G15-H15-I15-N15</f>
         <v/>
       </c>
       <c r="K15" s="109">
@@ -5014,6 +5114,10 @@
       </c>
       <c r="L15" s="98">
         <f>SUM($J$4:J15)</f>
+        <v/>
+      </c>
+      <c r="N15">
+        <f>IF(A15&lt;=12,Inputs!$B$36,IF(A15&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5054,7 +5158,7 @@
         <v/>
       </c>
       <c r="J16" s="98">
-        <f>E16-F16-G16-H16-I16</f>
+        <f>E16-F16-G16-H16-I16-N16</f>
         <v/>
       </c>
       <c r="K16" s="109">
@@ -5063,6 +5167,10 @@
       </c>
       <c r="L16" s="98">
         <f>SUM($J$4:J16)</f>
+        <v/>
+      </c>
+      <c r="N16">
+        <f>IF(A16&lt;=12,Inputs!$B$36,IF(A16&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5103,7 +5211,7 @@
         <v/>
       </c>
       <c r="J17" s="98">
-        <f>E17-F17-G17-H17-I17</f>
+        <f>E17-F17-G17-H17-I17-N17</f>
         <v/>
       </c>
       <c r="K17" s="109">
@@ -5112,6 +5220,10 @@
       </c>
       <c r="L17" s="98">
         <f>SUM($J$4:J17)</f>
+        <v/>
+      </c>
+      <c r="N17">
+        <f>IF(A17&lt;=12,Inputs!$B$36,IF(A17&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5152,7 +5264,7 @@
         <v/>
       </c>
       <c r="J18" s="98">
-        <f>E18-F18-G18-H18-I18</f>
+        <f>E18-F18-G18-H18-I18-N18</f>
         <v/>
       </c>
       <c r="K18" s="109">
@@ -5161,6 +5273,10 @@
       </c>
       <c r="L18" s="98">
         <f>SUM($J$4:J18)</f>
+        <v/>
+      </c>
+      <c r="N18">
+        <f>IF(A18&lt;=12,Inputs!$B$36,IF(A18&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5201,7 +5317,7 @@
         <v/>
       </c>
       <c r="J19" s="98">
-        <f>E19-F19-G19-H19-I19</f>
+        <f>E19-F19-G19-H19-I19-N19</f>
         <v/>
       </c>
       <c r="K19" s="109">
@@ -5210,6 +5326,10 @@
       </c>
       <c r="L19" s="98">
         <f>SUM($J$4:J19)</f>
+        <v/>
+      </c>
+      <c r="N19">
+        <f>IF(A19&lt;=12,Inputs!$B$36,IF(A19&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5250,7 +5370,7 @@
         <v/>
       </c>
       <c r="J20" s="98">
-        <f>E20-F20-G20-H20-I20</f>
+        <f>E20-F20-G20-H20-I20-N20</f>
         <v/>
       </c>
       <c r="K20" s="109">
@@ -5259,6 +5379,10 @@
       </c>
       <c r="L20" s="98">
         <f>SUM($J$4:J20)</f>
+        <v/>
+      </c>
+      <c r="N20">
+        <f>IF(A20&lt;=12,Inputs!$B$36,IF(A20&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5299,7 +5423,7 @@
         <v/>
       </c>
       <c r="J21" s="98">
-        <f>E21-F21-G21-H21-I21</f>
+        <f>E21-F21-G21-H21-I21-N21</f>
         <v/>
       </c>
       <c r="K21" s="109">
@@ -5308,6 +5432,10 @@
       </c>
       <c r="L21" s="98">
         <f>SUM($J$4:J21)</f>
+        <v/>
+      </c>
+      <c r="N21">
+        <f>IF(A21&lt;=12,Inputs!$B$36,IF(A21&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5348,7 +5476,7 @@
         <v/>
       </c>
       <c r="J22" s="98">
-        <f>E22-F22-G22-H22-I22</f>
+        <f>E22-F22-G22-H22-I22-N22</f>
         <v/>
       </c>
       <c r="K22" s="109">
@@ -5357,6 +5485,10 @@
       </c>
       <c r="L22" s="98">
         <f>SUM($J$4:J22)</f>
+        <v/>
+      </c>
+      <c r="N22">
+        <f>IF(A22&lt;=12,Inputs!$B$36,IF(A22&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5397,7 +5529,7 @@
         <v/>
       </c>
       <c r="J23" s="98">
-        <f>E23-F23-G23-H23-I23</f>
+        <f>E23-F23-G23-H23-I23-N23</f>
         <v/>
       </c>
       <c r="K23" s="109">
@@ -5406,6 +5538,10 @@
       </c>
       <c r="L23" s="98">
         <f>SUM($J$4:J23)</f>
+        <v/>
+      </c>
+      <c r="N23">
+        <f>IF(A23&lt;=12,Inputs!$B$36,IF(A23&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5446,7 +5582,7 @@
         <v/>
       </c>
       <c r="J24" s="98">
-        <f>E24-F24-G24-H24-I24</f>
+        <f>E24-F24-G24-H24-I24-N24</f>
         <v/>
       </c>
       <c r="K24" s="109">
@@ -5455,6 +5591,10 @@
       </c>
       <c r="L24" s="98">
         <f>SUM($J$4:J24)</f>
+        <v/>
+      </c>
+      <c r="N24">
+        <f>IF(A24&lt;=12,Inputs!$B$36,IF(A24&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5495,7 +5635,7 @@
         <v/>
       </c>
       <c r="J25" s="98">
-        <f>E25-F25-G25-H25-I25</f>
+        <f>E25-F25-G25-H25-I25-N25</f>
         <v/>
       </c>
       <c r="K25" s="109">
@@ -5504,6 +5644,10 @@
       </c>
       <c r="L25" s="98">
         <f>SUM($J$4:J25)</f>
+        <v/>
+      </c>
+      <c r="N25">
+        <f>IF(A25&lt;=12,Inputs!$B$36,IF(A25&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5544,7 +5688,7 @@
         <v/>
       </c>
       <c r="J26" s="98">
-        <f>E26-F26-G26-H26-I26</f>
+        <f>E26-F26-G26-H26-I26-N26</f>
         <v/>
       </c>
       <c r="K26" s="109">
@@ -5553,6 +5697,10 @@
       </c>
       <c r="L26" s="98">
         <f>SUM($J$4:J26)</f>
+        <v/>
+      </c>
+      <c r="N26">
+        <f>IF(A26&lt;=12,Inputs!$B$36,IF(A26&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5593,7 +5741,7 @@
         <v/>
       </c>
       <c r="J27" s="98">
-        <f>E27-F27-G27-H27-I27</f>
+        <f>E27-F27-G27-H27-I27-N27</f>
         <v/>
       </c>
       <c r="K27" s="109">
@@ -5602,6 +5750,10 @@
       </c>
       <c r="L27" s="98">
         <f>SUM($J$4:J27)</f>
+        <v/>
+      </c>
+      <c r="N27">
+        <f>IF(A27&lt;=12,Inputs!$B$36,IF(A27&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5642,7 +5794,7 @@
         <v/>
       </c>
       <c r="J28" s="98">
-        <f>E28-F28-G28-H28-I28</f>
+        <f>E28-F28-G28-H28-I28-N28</f>
         <v/>
       </c>
       <c r="K28" s="109">
@@ -5651,6 +5803,10 @@
       </c>
       <c r="L28" s="98">
         <f>SUM($J$4:J28)</f>
+        <v/>
+      </c>
+      <c r="N28">
+        <f>IF(A28&lt;=12,Inputs!$B$36,IF(A28&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5691,7 +5847,7 @@
         <v/>
       </c>
       <c r="J29" s="98">
-        <f>E29-F29-G29-H29-I29</f>
+        <f>E29-F29-G29-H29-I29-N29</f>
         <v/>
       </c>
       <c r="K29" s="109">
@@ -5700,6 +5856,10 @@
       </c>
       <c r="L29" s="98">
         <f>SUM($J$4:J29)</f>
+        <v/>
+      </c>
+      <c r="N29">
+        <f>IF(A29&lt;=12,Inputs!$B$36,IF(A29&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5740,7 +5900,7 @@
         <v/>
       </c>
       <c r="J30" s="98">
-        <f>E30-F30-G30-H30-I30</f>
+        <f>E30-F30-G30-H30-I30-N30</f>
         <v/>
       </c>
       <c r="K30" s="109">
@@ -5749,6 +5909,10 @@
       </c>
       <c r="L30" s="98">
         <f>SUM($J$4:J30)</f>
+        <v/>
+      </c>
+      <c r="N30">
+        <f>IF(A30&lt;=12,Inputs!$B$36,IF(A30&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5789,7 +5953,7 @@
         <v/>
       </c>
       <c r="J31" s="98">
-        <f>E31-F31-G31-H31-I31</f>
+        <f>E31-F31-G31-H31-I31-N31</f>
         <v/>
       </c>
       <c r="K31" s="109">
@@ -5798,6 +5962,10 @@
       </c>
       <c r="L31" s="98">
         <f>SUM($J$4:J31)</f>
+        <v/>
+      </c>
+      <c r="N31">
+        <f>IF(A31&lt;=12,Inputs!$B$36,IF(A31&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5838,7 +6006,7 @@
         <v/>
       </c>
       <c r="J32" s="98">
-        <f>E32-F32-G32-H32-I32</f>
+        <f>E32-F32-G32-H32-I32-N32</f>
         <v/>
       </c>
       <c r="K32" s="109">
@@ -5847,6 +6015,10 @@
       </c>
       <c r="L32" s="98">
         <f>SUM($J$4:J32)</f>
+        <v/>
+      </c>
+      <c r="N32">
+        <f>IF(A32&lt;=12,Inputs!$B$36,IF(A32&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5887,7 +6059,7 @@
         <v/>
       </c>
       <c r="J33" s="98">
-        <f>E33-F33-G33-H33-I33</f>
+        <f>E33-F33-G33-H33-I33-N33</f>
         <v/>
       </c>
       <c r="K33" s="109">
@@ -5896,6 +6068,10 @@
       </c>
       <c r="L33" s="98">
         <f>SUM($J$4:J33)</f>
+        <v/>
+      </c>
+      <c r="N33">
+        <f>IF(A33&lt;=12,Inputs!$B$36,IF(A33&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5936,7 +6112,7 @@
         <v/>
       </c>
       <c r="J34" s="98">
-        <f>E34-F34-G34-H34-I34</f>
+        <f>E34-F34-G34-H34-I34-N34</f>
         <v/>
       </c>
       <c r="K34" s="109">
@@ -5945,6 +6121,10 @@
       </c>
       <c r="L34" s="98">
         <f>SUM($J$4:J34)</f>
+        <v/>
+      </c>
+      <c r="N34">
+        <f>IF(A34&lt;=12,Inputs!$B$36,IF(A34&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -5985,7 +6165,7 @@
         <v/>
       </c>
       <c r="J35" s="98">
-        <f>E35-F35-G35-H35-I35</f>
+        <f>E35-F35-G35-H35-I35-N35</f>
         <v/>
       </c>
       <c r="K35" s="109">
@@ -5994,6 +6174,10 @@
       </c>
       <c r="L35" s="98">
         <f>SUM($J$4:J35)</f>
+        <v/>
+      </c>
+      <c r="N35">
+        <f>IF(A35&lt;=12,Inputs!$B$36,IF(A35&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -6034,7 +6218,7 @@
         <v/>
       </c>
       <c r="J36" s="98">
-        <f>E36-F36-G36-H36-I36</f>
+        <f>E36-F36-G36-H36-I36-N36</f>
         <v/>
       </c>
       <c r="K36" s="109">
@@ -6043,6 +6227,10 @@
       </c>
       <c r="L36" s="98">
         <f>SUM($J$4:J36)</f>
+        <v/>
+      </c>
+      <c r="N36">
+        <f>IF(A36&lt;=12,Inputs!$B$36,IF(A36&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -6083,7 +6271,7 @@
         <v/>
       </c>
       <c r="J37" s="98">
-        <f>E37-F37-G37-H37-I37</f>
+        <f>E37-F37-G37-H37-I37-N37</f>
         <v/>
       </c>
       <c r="K37" s="109">
@@ -6092,6 +6280,10 @@
       </c>
       <c r="L37" s="98">
         <f>SUM($J$4:J37)</f>
+        <v/>
+      </c>
+      <c r="N37">
+        <f>IF(A37&lt;=12,Inputs!$B$36,IF(A37&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -6132,7 +6324,7 @@
         <v/>
       </c>
       <c r="J38" s="98">
-        <f>E38-F38-G38-H38-I38</f>
+        <f>E38-F38-G38-H38-I38-N38</f>
         <v/>
       </c>
       <c r="K38" s="109">
@@ -6141,6 +6333,10 @@
       </c>
       <c r="L38" s="98">
         <f>SUM($J$4:J38)</f>
+        <v/>
+      </c>
+      <c r="N38">
+        <f>IF(A38&lt;=12,Inputs!$B$36,IF(A38&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -6181,7 +6377,7 @@
         <v/>
       </c>
       <c r="J39" s="98">
-        <f>E39-F39-G39-H39-I39</f>
+        <f>E39-F39-G39-H39-I39-N39</f>
         <v/>
       </c>
       <c r="K39" s="109">
@@ -6190,6 +6386,10 @@
       </c>
       <c r="L39" s="98">
         <f>SUM($J$4:J39)</f>
+        <v/>
+      </c>
+      <c r="N39">
+        <f>IF(A39&lt;=12,Inputs!$B$36,IF(A39&lt;=24,Inputs!$B$37,Inputs!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -8092,15 +8292,15 @@
         </is>
       </c>
       <c r="B7" s="98">
-        <f>(Socios_36M!B$39*(Inputs!B$27+Inputs!B$28)/(1+Inputs!$B$12)-Socios_36M!B$39*Inputs!B$29-Inputs!$B$16-Inputs!$B$17-Inputs!B$30)*12</f>
+        <f>(Socios_36M!B$39*(Inputs!B$27+Inputs!B$28)/(1+Inputs!$B$12)-Socios_36M!B$39*Inputs!B$29-Inputs!$B$16-Inputs!$B$17-Inputs!B$30-Inputs!$B$38)*12</f>
         <v/>
       </c>
       <c r="C7" s="98">
-        <f>(Socios_36M!C$39*(Inputs!C$27+Inputs!C$28)/(1+Inputs!$B$12)-Socios_36M!C$39*Inputs!C$29-Inputs!$B$16-Inputs!$B$17-Inputs!C$30)*12</f>
+        <f>(Socios_36M!C$39*(Inputs!C$27+Inputs!C$28)/(1+Inputs!$B$12)-Socios_36M!C$39*Inputs!C$29-Inputs!$B$16-Inputs!$B$17-Inputs!C$30-Inputs!$B$38)*12</f>
         <v/>
       </c>
       <c r="D7" s="98">
-        <f>(Socios_36M!D$39*(Inputs!D$27+Inputs!D$28)/(1+Inputs!$B$12)-Socios_36M!D$39*Inputs!D$29-Inputs!$B$16-Inputs!$B$17-Inputs!D$30)*12</f>
+        <f>(Socios_36M!D$39*(Inputs!D$27+Inputs!D$28)/(1+Inputs!$B$12)-Socios_36M!D$39*Inputs!D$29-Inputs!$B$16-Inputs!$B$17-Inputs!D$30-Inputs!$B$38)*12</f>
         <v/>
       </c>
       <c r="E7" t="inlineStr">
@@ -8346,7 +8546,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sergi / fundador</t>
+          <t>Sergi Caro Folch</t>
         </is>
       </c>
       <c r="B4" s="102" t="n">
@@ -8374,14 +8574,14 @@
       </c>
       <c r="H4" s="38" t="inlineStr">
         <is>
-          <t>Ejemplo editable: sustituir por reparto real.</t>
+          <t>Socio fundador, 20% cada uno (a validar con escritura real).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marta</t>
+          <t>Marta Folch Gorina</t>
         </is>
       </c>
       <c r="B5" s="102" t="n">
@@ -8409,14 +8609,14 @@
       </c>
       <c r="H5" s="38" t="inlineStr">
         <is>
-          <t>Ejemplo editable.</t>
+          <t>Socio fundador, 20% cada uno (a validar con escritura real).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>Antonio Caro</t>
         </is>
       </c>
       <c r="B6" s="102" t="n">
@@ -8444,14 +8644,14 @@
       </c>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>Ejemplo editable.</t>
+          <t>Socio fundador, 20% cada uno (a validar con escritura real).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arnau</t>
+          <t>Arnau Caro Folch</t>
         </is>
       </c>
       <c r="B7" s="102" t="n">
@@ -8479,14 +8679,14 @@
       </c>
       <c r="H7" s="38" t="inlineStr">
         <is>
-          <t>Ejemplo editable.</t>
+          <t>Socio fundador, 20% cada uno (a validar con escritura real).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Óscar</t>
+          <t>Óscar Caro Folch</t>
         </is>
       </c>
       <c r="B8" s="102" t="n">
@@ -8514,7 +8714,7 @@
       </c>
       <c r="H8" s="38" t="inlineStr">
         <is>
-          <t>Ejemplo editable.</t>
+          <t>Socio fundador, 20% cada uno (a validar con escritura real).</t>
         </is>
       </c>
     </row>

</xml_diff>